<commit_message>
feat: add environment computer and report fees
</commit_message>
<xml_diff>
--- a/outputs/mla-fee-detail-export/JLR- MLA 费用规则.xlsx
+++ b/outputs/mla-fee-detail-export/JLR- MLA 费用规则.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28180" windowHeight="12560" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="费用规则去重表" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="费用规则去重表" sheetId="1" state="visible" ns1:id="rId1"/>
+    <sheet name="版本记录" sheetId="2" state="visible" ns1:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'费用规则去重表'!$A$1:$AC$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'版本记录'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'费用规则去重表'!$A$1:$AD$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'版本记录'!$A$1:$F$3</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -1307,7 +1307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD34"/>
+  <dimension ref="A1:AD36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.2"/>
   <cols>
     <col width="15" customWidth="1" style="3" min="1" max="1"/>
@@ -4761,10 +4761,234 @@
         </is>
       </c>
     </row>
+    <row r="35" ht="46" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Computer Fee</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Computer Fee</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Computer Fee</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>委外费用</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>按月/台计费</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>computerCoefficient</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="H35" s="6">
+        <f>IF(G35="","",IF(G35&lt;=6,"小环境箱","大环境箱"))</f>
+      </c>
+      <c r="I35" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>系数默认 48，可在页面展开后人工修改</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="M35" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="N35" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="O35" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="P35" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="Q35" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="R35" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="S35" s="7" t="n">
+        <v>12000</v>
+      </c>
+      <c r="T35" s="7" t="n">
+        <v>450</v>
+      </c>
+      <c r="U35" s="7" t="n">
+        <v>21600</v>
+      </c>
+      <c r="V35" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="W35" s="7" t="n">
+        <v>7200</v>
+      </c>
+      <c r="X35" s="7">
+        <f>S35</f>
+      </c>
+      <c r="Y35" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="Z35" s="8">
+        <f>IF(Y35&lt;&gt;"",Y35,X35)</f>
+      </c>
+      <c r="AA35" s="9" t="inlineStr">
+        <is>
+          <t>SGS: 250/月/台 × 48 = 12000；华测: 450/月/台 × 48 = 21600；苏勃: 150/月/台 × 48 = 7200</t>
+        </is>
+      </c>
+      <c r="AB35" s="5" t="inlineStr">
+        <is>
+          <t>电脑费用计入顶部 Total Cost；当前按 SGS 报价计入，系数默认 48，可编辑。</t>
+        </is>
+      </c>
+      <c r="AC35" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD35" s="3" t="inlineStr">
+        <is/>
+      </c>
+    </row>
+    <row r="36" ht="46" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Report Fee</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Report Fee</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Report Fee</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>委外费用</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>按报告份数计费/份</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>reportCount</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="H36" s="6">
+        <f>IF(G36="","",IF(G36&lt;=6,"小环境箱","大环境箱"))</f>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>默认按当前 phase 实际组数量，每组一份；本规则表示例按 DV 13 组</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="M36" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="N36" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="O36" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="P36" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="Q36" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="R36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="W36" s="7" t="n">
+        <v>1950</v>
+      </c>
+      <c r="X36" s="7">
+        <f>W36</f>
+      </c>
+      <c r="Y36" s="6" t="inlineStr">
+        <is/>
+      </c>
+      <c r="Z36" s="8">
+        <f>IF(Y36&lt;&gt;"",Y36,X36)</f>
+      </c>
+      <c r="AA36" s="9" t="inlineStr">
+        <is>
+          <t>SGS: 0/份 × 13 份 = 0；华测: 0/份 × 13 份 = 0；苏勃: 150/份 × 13 份 = 1950</t>
+        </is>
+      </c>
+      <c r="AB36" s="5" t="inlineStr">
+        <is>
+          <t>报告费用计入顶部 Total Cost；SGS/华测为 0，当前按苏勃 150/份计入；报告份数默认每组一份，可编辑。</t>
+        </is>
+      </c>
+      <c r="AC36" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD36" s="3" t="inlineStr">
+        <is/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AC34"/>
+  <autoFilter ref="A1:AD36"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2 D3 D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31:D34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"内部费用,委外费用,内外部都可,待确认"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4778,7 +5002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.2" outlineLevelRow="1"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4853,8 +5077,40 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="58" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>V.1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>费用规则补充</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>新增顶部附加费用规则：Computer Fee 按实验室月/台单价 × 系数计算，默认系数 48，当前按 SGS 计入；Report Fee 按实验室每份报告单价 × 报告份数计算，默认每组一份，当前按苏勃 150/份计入；Total Cost 口径同步为各组测试费用 + Computer Fee + Report Fee。</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>费用规则去重表；/environment-outline 顶部费用汇总</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>对应系统本地草稿模板版本 ENVIRONMENT_PLAN_TEMPLATE_VERSION = 36。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F2"/>
+  <autoFilter ref="A1:F3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>